<commit_message>
Set GLP3-R powder price to $10 per mg
5mg $50, 10mg $100, 15mg $150, 20mg $200, 30mg $300, 50mg $500.
Ready-to-use follows via the existing powder + 20% rule.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/price_list_source.xlsx
+++ b/data/price_list_source.xlsx
@@ -1831,7 +1831,7 @@
         <v>6</v>
       </c>
       <c r="D11" s="9">
-        <v>80.0</v>
+        <v>50.0</v>
       </c>
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
@@ -1865,7 +1865,7 @@
         <v>8</v>
       </c>
       <c r="D12" s="9">
-        <v>90.0</v>
+        <v>100.0</v>
       </c>
       <c r="E12" s="5"/>
       <c r="F12" s="5"/>
@@ -1899,7 +1899,7 @@
         <v>10</v>
       </c>
       <c r="D13" s="13">
-        <v>110.0</v>
+        <v>150.0</v>
       </c>
       <c r="E13" s="5"/>
       <c r="F13" s="5"/>
@@ -1933,7 +1933,7 @@
         <v>12</v>
       </c>
       <c r="D14" s="13">
-        <v>145.0</v>
+        <v>200.0</v>
       </c>
       <c r="E14" s="5"/>
       <c r="F14" s="5"/>
@@ -1967,7 +1967,7 @@
         <v>14</v>
       </c>
       <c r="D15" s="13">
-        <v>190.0</v>
+        <v>300.0</v>
       </c>
       <c r="E15" s="5"/>
       <c r="F15" s="5"/>
@@ -2001,7 +2001,7 @@
         <v>20</v>
       </c>
       <c r="D16" s="13">
-        <v>320.0</v>
+        <v>500.0</v>
       </c>
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>

</xml_diff>